<commit_message>
fix: corriger la fuite de donnees statut_prevu/priorite_recommandee
- exclure les 2 colonnes fuyantes (corr 0.85/0.83 avec la cible) du pipeline ML
- notebook 07 reexecute sans fuite : baseline honnete R2 ~0.30, LightGBM optimise R2 0.2986
- retrainer le modele deploye en LightGBM optimise (46 features, plus de fuite)
- regenerer dashboard, importances et metriques (suppression des anciens R2 0.775/0.833)
- ajouter lightgbm et seaborn a requirements.txt
</commit_message>
<xml_diff>
--- a/results/comparaison_modeles.xlsx
+++ b/results/comparaison_modeles.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,41 +413,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Modele</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>MAE</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>RMSE</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>MAPE</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Temps_Entrainement</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Temps_Prediction</t>
         </is>
@@ -468,151 +456,172 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Gradient Boosting</t>
+          <t>LightGBM optimisé (déployé)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6.311118566238268</v>
+        <v>11.579088</v>
       </c>
       <c r="C2" t="n">
-        <v>8.056672354383727</v>
+        <v>15.442533</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6752653621682901</v>
+        <v>115.768809</v>
       </c>
       <c r="E2" t="n">
-        <v>0.7752168834494355</v>
-      </c>
-      <c r="F2" t="n">
-        <v>83.25329995155334</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0.1083741188049316</v>
-      </c>
+        <v>0.298569</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>LightGBM</t>
+          <t>CatBoost</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>6.242009444122437</v>
+        <v>11.60395568531778</v>
       </c>
       <c r="C3" t="n">
-        <v>8.056756582724322</v>
+        <v>15.45615909556452</v>
       </c>
       <c r="D3" t="n">
-        <v>0.6726236816232064</v>
+        <v>116.0827329808902</v>
       </c>
       <c r="E3" t="n">
-        <v>0.7752121834425254</v>
+        <v>0.2973301876884507</v>
       </c>
       <c r="F3" t="n">
-        <v>1.247756004333496</v>
+        <v>6.351865768432617</v>
       </c>
       <c r="G3" t="n">
-        <v>0.04154586791992188</v>
+        <v>0.02170896530151367</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CatBoost</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6.242235868732825</v>
+        <v>11.49366746152182</v>
       </c>
       <c r="C4" t="n">
-        <v>8.085187316817235</v>
+        <v>15.47542749316548</v>
       </c>
       <c r="D4" t="n">
-        <v>0.6769788374369226</v>
+        <v>115.2407145428648</v>
       </c>
       <c r="E4" t="n">
-        <v>0.7736229189120962</v>
+        <v>0.2955771311070087</v>
       </c>
       <c r="F4" t="n">
-        <v>23.46304941177368</v>
+        <v>3.567641973495483</v>
       </c>
       <c r="G4" t="n">
-        <v>0.02562642097473145</v>
+        <v>0.08769011497497559</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Random Forest</t>
+          <t>LightGBM</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6.304479203721791</v>
+        <v>11.53490787664372</v>
       </c>
       <c r="C5" t="n">
-        <v>8.100404915721867</v>
+        <v>15.47935711798879</v>
       </c>
       <c r="D5" t="n">
-        <v>0.6721213142396855</v>
+        <v>115.4919540210417</v>
       </c>
       <c r="E5" t="n">
-        <v>0.7727699621595565</v>
+        <v>0.2952193420840602</v>
       </c>
       <c r="F5" t="n">
-        <v>256.0675117969513</v>
+        <v>2.766029357910156</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4878537654876709</v>
+        <v>0.1276133060455322</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Gradient Boosting</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6.396908266476014</v>
+        <v>11.65499769032685</v>
       </c>
       <c r="C6" t="n">
-        <v>8.285991393817985</v>
+        <v>15.48430731452359</v>
       </c>
       <c r="D6" t="n">
-        <v>0.6724071711860081</v>
+        <v>116.3301502410612</v>
       </c>
       <c r="E6" t="n">
-        <v>0.7622386601326138</v>
+        <v>0.2947685015753631</v>
       </c>
       <c r="F6" t="n">
-        <v>1.569111347198486</v>
+        <v>247.9452774524689</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0378413200378418</v>
+        <v>0.2030115127563477</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>11.6844971489726</v>
+      </c>
+      <c r="C7" t="n">
+        <v>15.74748451117665</v>
+      </c>
+      <c r="D7" t="n">
+        <v>115.4768627872369</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.2705920090304367</v>
+      </c>
+      <c r="F7" t="n">
+        <v>260.9399950504303</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.831757783889771</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Linear Regression</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>7.911781093746022</v>
-      </c>
-      <c r="C7" t="n">
-        <v>9.448653865784989</v>
-      </c>
-      <c r="D7" t="n">
-        <v>0.7400711722030481</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.6908336896048177</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0.2925708293914795</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.01331973075866699</v>
+      <c r="B8" t="n">
+        <v>11.9813644297274</v>
+      </c>
+      <c r="C8" t="n">
+        <v>15.77056878169202</v>
+      </c>
+      <c r="D8" t="n">
+        <v>118.7201554636265</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.268451960226013</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.4423985481262207</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.05148172378540039</v>
       </c>
     </row>
   </sheetData>

</xml_diff>